<commit_message>
Fix SHORT_CODES word boundary bug, add Honda/GEELY car brand maps, handle model aliases (MEGANESD, 207HB, etc), improve first_model_word for numeric models, add car/moto fallback matching - 98.8% success rate (337/341)
</commit_message>
<xml_diff>
--- a/lotes_leilao_com_fipe.xlsx
+++ b/lotes_leilao_com_fipe.xlsx
@@ -728,7 +728,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 7.049,00</t>
         </is>
       </c>
     </row>
@@ -840,7 +840,7 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 6.377,00</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 22.412,00</t>
         </is>
       </c>
     </row>
@@ -1652,7 +1652,7 @@
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 7.738,00</t>
         </is>
       </c>
     </row>
@@ -1680,7 +1680,7 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 8.637,00</t>
         </is>
       </c>
     </row>
@@ -2772,7 +2772,7 @@
       </c>
       <c r="F82" t="inlineStr">
         <is>
-          <t>R$ 66.738,00</t>
+          <t>R$ 33.985,00</t>
         </is>
       </c>
     </row>
@@ -3115,7 +3115,7 @@
       </c>
       <c r="F95" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 22.412,00</t>
         </is>
       </c>
     </row>
@@ -3143,7 +3143,7 @@
       </c>
       <c r="F96" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 7.232,00</t>
         </is>
       </c>
     </row>
@@ -3171,7 +3171,7 @@
       </c>
       <c r="F97" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 10.295,00</t>
         </is>
       </c>
     </row>
@@ -3199,7 +3199,7 @@
       </c>
       <c r="F98" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 8.484,00</t>
         </is>
       </c>
     </row>
@@ -3227,7 +3227,7 @@
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 6.217,00</t>
         </is>
       </c>
     </row>
@@ -3283,7 +3283,7 @@
       </c>
       <c r="F101" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 7.120,00</t>
         </is>
       </c>
     </row>
@@ -3339,7 +3339,7 @@
       </c>
       <c r="F103" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 2.605,00</t>
         </is>
       </c>
     </row>
@@ -3367,7 +3367,7 @@
       </c>
       <c r="F104" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 22.412,00</t>
         </is>
       </c>
     </row>
@@ -3423,7 +3423,7 @@
       </c>
       <c r="F106" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 7.669,00</t>
         </is>
       </c>
     </row>
@@ -3479,7 +3479,7 @@
       </c>
       <c r="F108" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 5.892,00</t>
         </is>
       </c>
     </row>
@@ -3507,7 +3507,7 @@
       </c>
       <c r="F109" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 15.712,00</t>
         </is>
       </c>
     </row>
@@ -3563,7 +3563,7 @@
       </c>
       <c r="F111" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 7.669,00</t>
         </is>
       </c>
     </row>
@@ -3619,7 +3619,7 @@
       </c>
       <c r="F113" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 16.472,00</t>
         </is>
       </c>
     </row>
@@ -3703,7 +3703,7 @@
       </c>
       <c r="F116" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 7.368,00</t>
         </is>
       </c>
     </row>
@@ -3759,7 +3759,7 @@
       </c>
       <c r="F118" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 3.279,00</t>
         </is>
       </c>
     </row>
@@ -3843,7 +3843,7 @@
       </c>
       <c r="F121" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 4.608,00</t>
         </is>
       </c>
     </row>
@@ -3871,7 +3871,7 @@
       </c>
       <c r="F122" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 7.235,00</t>
         </is>
       </c>
     </row>
@@ -3899,7 +3899,7 @@
       </c>
       <c r="F123" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 16.357,00</t>
         </is>
       </c>
     </row>
@@ -3955,7 +3955,7 @@
       </c>
       <c r="F125" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 7.878,00</t>
         </is>
       </c>
     </row>
@@ -3983,7 +3983,7 @@
       </c>
       <c r="F126" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 4.540,00</t>
         </is>
       </c>
     </row>
@@ -4067,7 +4067,7 @@
       </c>
       <c r="F129" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 9.693,00</t>
         </is>
       </c>
     </row>
@@ -4123,7 +4123,7 @@
       </c>
       <c r="F131" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 7.368,00</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="F132" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 8.972,00</t>
         </is>
       </c>
     </row>
@@ -4207,7 +4207,7 @@
       </c>
       <c r="F134" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 4.122,00</t>
         </is>
       </c>
     </row>
@@ -4235,7 +4235,7 @@
       </c>
       <c r="F135" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 7.425,00</t>
         </is>
       </c>
     </row>
@@ -4319,7 +4319,7 @@
       </c>
       <c r="F138" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 8.079,00</t>
         </is>
       </c>
     </row>
@@ -4375,7 +4375,7 @@
       </c>
       <c r="F140" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 22.412,00</t>
         </is>
       </c>
     </row>
@@ -4403,7 +4403,7 @@
       </c>
       <c r="F141" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 21.691,00</t>
         </is>
       </c>
     </row>
@@ -4431,7 +4431,7 @@
       </c>
       <c r="F142" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 6.217,00</t>
         </is>
       </c>
     </row>
@@ -4459,7 +4459,7 @@
       </c>
       <c r="F143" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 8.653,00</t>
         </is>
       </c>
     </row>
@@ -4571,7 +4571,7 @@
       </c>
       <c r="F147" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 9.946,00</t>
         </is>
       </c>
     </row>
@@ -4599,7 +4599,7 @@
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 9.442,00</t>
         </is>
       </c>
     </row>
@@ -4627,7 +4627,7 @@
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 9.949,00</t>
         </is>
       </c>
     </row>
@@ -4655,7 +4655,7 @@
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 3.727,00</t>
         </is>
       </c>
     </row>
@@ -4683,7 +4683,7 @@
       </c>
       <c r="F151" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 9.950,00</t>
         </is>
       </c>
     </row>
@@ -4711,7 +4711,7 @@
       </c>
       <c r="F152" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 9.671,00</t>
         </is>
       </c>
     </row>
@@ -5159,7 +5159,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 14.836,00</t>
         </is>
       </c>
     </row>
@@ -5187,7 +5187,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 14.825,00</t>
         </is>
       </c>
     </row>
@@ -5327,7 +5327,7 @@
       </c>
       <c r="F174" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 30.112,00</t>
         </is>
       </c>
     </row>
@@ -5775,7 +5775,7 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>R$ 15.161,00</t>
+          <t>R$ 7.962,00</t>
         </is>
       </c>
     </row>
@@ -5859,7 +5859,7 @@
       </c>
       <c r="F193" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 31.972,00</t>
         </is>
       </c>
     </row>
@@ -6027,7 +6027,7 @@
       </c>
       <c r="F199" t="inlineStr">
         <is>
-          <t>R$ 7.899,00</t>
+          <t>R$ 23.496,00</t>
         </is>
       </c>
     </row>
@@ -6363,7 +6363,7 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 17.829,00</t>
         </is>
       </c>
     </row>
@@ -6699,7 +6699,7 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 9.544,00</t>
         </is>
       </c>
     </row>
@@ -7063,7 +7063,7 @@
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 52.240,00</t>
         </is>
       </c>
     </row>
@@ -7434,7 +7434,7 @@
       </c>
       <c r="F250" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 7.669,00</t>
         </is>
       </c>
     </row>
@@ -7462,7 +7462,7 @@
       </c>
       <c r="F251" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 7.878,00</t>
         </is>
       </c>
     </row>
@@ -7546,7 +7546,7 @@
       </c>
       <c r="F254" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 3.041,00</t>
         </is>
       </c>
     </row>
@@ -7574,7 +7574,7 @@
       </c>
       <c r="F255" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 22.412,00</t>
         </is>
       </c>
     </row>
@@ -7602,7 +7602,7 @@
       </c>
       <c r="F256" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 7.368,00</t>
         </is>
       </c>
     </row>
@@ -7658,7 +7658,7 @@
       </c>
       <c r="F258" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 6.325,00</t>
         </is>
       </c>
     </row>
@@ -7742,7 +7742,7 @@
       </c>
       <c r="F261" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 7.476,00</t>
         </is>
       </c>
     </row>
@@ -7770,7 +7770,7 @@
       </c>
       <c r="F262" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 6.705,00</t>
         </is>
       </c>
     </row>
@@ -7882,7 +7882,7 @@
       </c>
       <c r="F266" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 8.317,00</t>
         </is>
       </c>
     </row>
@@ -7938,7 +7938,7 @@
       </c>
       <c r="F268" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 6.873,00</t>
         </is>
       </c>
     </row>
@@ -7966,7 +7966,7 @@
       </c>
       <c r="F269" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 14.494,00</t>
         </is>
       </c>
     </row>
@@ -7994,7 +7994,7 @@
       </c>
       <c r="F270" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 7.232,00</t>
         </is>
       </c>
     </row>
@@ -8078,7 +8078,7 @@
       </c>
       <c r="F273" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 9.553,00</t>
         </is>
       </c>
     </row>
@@ -8106,7 +8106,7 @@
       </c>
       <c r="F274" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 8.484,00</t>
         </is>
       </c>
     </row>
@@ -8218,7 +8218,7 @@
       </c>
       <c r="F278" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 2.092,00</t>
         </is>
       </c>
     </row>
@@ -8246,7 +8246,7 @@
       </c>
       <c r="F279" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 2.237,00</t>
         </is>
       </c>
     </row>
@@ -8274,7 +8274,7 @@
       </c>
       <c r="F280" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 7.669,00</t>
         </is>
       </c>
     </row>
@@ -8330,7 +8330,7 @@
       </c>
       <c r="F282" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 7.800,00</t>
         </is>
       </c>
     </row>
@@ -8358,7 +8358,7 @@
       </c>
       <c r="F283" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 16.108,00</t>
         </is>
       </c>
     </row>
@@ -8386,7 +8386,7 @@
       </c>
       <c r="F284" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 9.946,00</t>
         </is>
       </c>
     </row>
@@ -8442,7 +8442,7 @@
       </c>
       <c r="F286" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 5.234,00</t>
         </is>
       </c>
     </row>
@@ -8498,7 +8498,7 @@
       </c>
       <c r="F288" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 8.484,00</t>
         </is>
       </c>
     </row>
@@ -8554,7 +8554,7 @@
       </c>
       <c r="F290" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 6.957,00</t>
         </is>
       </c>
     </row>
@@ -8582,7 +8582,7 @@
       </c>
       <c r="F291" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 13.803,00</t>
         </is>
       </c>
     </row>
@@ -8610,7 +8610,7 @@
       </c>
       <c r="F292" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 16.472,00</t>
         </is>
       </c>
     </row>
@@ -8694,7 +8694,7 @@
       </c>
       <c r="F295" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 8.525,00</t>
         </is>
       </c>
     </row>
@@ -8722,7 +8722,7 @@
       </c>
       <c r="F296" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 7.669,00</t>
         </is>
       </c>
     </row>
@@ -8750,7 +8750,7 @@
       </c>
       <c r="F297" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 14.311,00</t>
         </is>
       </c>
     </row>
@@ -8778,7 +8778,7 @@
       </c>
       <c r="F298" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 15.712,00</t>
         </is>
       </c>
     </row>
@@ -8806,7 +8806,7 @@
       </c>
       <c r="F299" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 6.500,00</t>
         </is>
       </c>
     </row>
@@ -8834,7 +8834,7 @@
       </c>
       <c r="F300" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 6.705,00</t>
         </is>
       </c>
     </row>
@@ -8862,7 +8862,7 @@
       </c>
       <c r="F301" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 8.293,00</t>
         </is>
       </c>
     </row>
@@ -8918,7 +8918,7 @@
       </c>
       <c r="F303" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 9.919,00</t>
         </is>
       </c>
     </row>
@@ -9002,7 +9002,7 @@
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>R$ 6.480,00</t>
+          <t>R$ 7.899,00</t>
         </is>
       </c>
     </row>
@@ -9478,7 +9478,7 @@
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>NAO ENCONTRADO</t>
+          <t>R$ 9.544,00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Major accuracy improvement: exclude commercial variants (Furgao), year-aware model scoring, trim-level matching (GL/CL/Life/Spirit/Maxx), combined scoring with displacement and year bonuses
Fixes: GOL->Gol Furgao (was R$6K, now R$24K correct), VOYAGE GL->GL/Special (was R$22K, now R$11K), CLASSIC LIFE year (was R$33K for 2016, now R$17K for 2005), CORSA HATCH MAXX variant (was R$32K 1.4, now R$18K 1.0)
</commit_message>
<xml_diff>
--- a/lotes_leilao_com_fipe.xlsx
+++ b/lotes_leilao_com_fipe.xlsx
@@ -1848,7 +1848,7 @@
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>R$ 14.608,00</t>
+          <t>R$ 18.112,00</t>
         </is>
       </c>
     </row>
@@ -1876,7 +1876,7 @@
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>R$ 10.464,00</t>
+          <t>R$ 29.850,00</t>
         </is>
       </c>
     </row>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>R$ 34.123,00</t>
+          <t>R$ 26.597,00</t>
         </is>
       </c>
     </row>
@@ -1960,7 +1960,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>R$ 6.505,00</t>
+          <t>R$ 8.553,00</t>
         </is>
       </c>
     </row>
@@ -1988,7 +1988,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>R$ 6.505,00</t>
+          <t>R$ 18.298,00</t>
         </is>
       </c>
     </row>
@@ -2072,7 +2072,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>R$ 6.505,00</t>
+          <t>R$ 8.553,00</t>
         </is>
       </c>
     </row>
@@ -2100,7 +2100,7 @@
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>R$ 6.505,00</t>
+          <t>R$ 23.869,00</t>
         </is>
       </c>
     </row>
@@ -2184,7 +2184,7 @@
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>R$ 6.505,00</t>
+          <t>R$ 27.806,00</t>
         </is>
       </c>
     </row>
@@ -2268,7 +2268,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>R$ 13.305,00</t>
+          <t>R$ 8.588,00</t>
         </is>
       </c>
     </row>
@@ -2296,7 +2296,7 @@
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>R$ 22.420,00</t>
+          <t>R$ 11.255,00</t>
         </is>
       </c>
     </row>
@@ -2324,7 +2324,7 @@
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>R$ 14.608,00</t>
+          <t>R$ 12.503,00</t>
         </is>
       </c>
     </row>
@@ -2352,7 +2352,7 @@
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>R$ 15.542,00</t>
+          <t>R$ 11.233,00</t>
         </is>
       </c>
     </row>
@@ -2380,7 +2380,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>R$ 6.505,00</t>
+          <t>R$ 24.466,00</t>
         </is>
       </c>
     </row>
@@ -2436,7 +2436,7 @@
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>R$ 13.598,00</t>
+          <t>R$ 10.216,00</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="F72" t="inlineStr">
         <is>
-          <t>R$ 8.635,00</t>
+          <t>R$ 18.974,00</t>
         </is>
       </c>
     </row>
@@ -2520,7 +2520,7 @@
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>R$ 28.002,00</t>
+          <t>R$ 27.246,00</t>
         </is>
       </c>
     </row>
@@ -2576,7 +2576,7 @@
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>R$ 34.123,00</t>
+          <t>R$ 21.648,00</t>
         </is>
       </c>
     </row>
@@ -2604,7 +2604,7 @@
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>R$ 13.309,00</t>
+          <t>R$ 16.436,00</t>
         </is>
       </c>
     </row>
@@ -2716,7 +2716,7 @@
       </c>
       <c r="F80" t="inlineStr">
         <is>
-          <t>R$ 119.907,00</t>
+          <t>R$ 51.260,00</t>
         </is>
       </c>
     </row>
@@ -2744,7 +2744,7 @@
       </c>
       <c r="F81" t="inlineStr">
         <is>
-          <t>R$ 29.261,00</t>
+          <t>R$ 10.236,00</t>
         </is>
       </c>
     </row>
@@ -2828,7 +2828,7 @@
       </c>
       <c r="F84" t="inlineStr">
         <is>
-          <t>R$ 6.505,00</t>
+          <t>R$ 24.466,00</t>
         </is>
       </c>
     </row>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="F87" t="inlineStr">
         <is>
-          <t>R$ 14.608,00</t>
+          <t>R$ 34.107,00</t>
         </is>
       </c>
     </row>
@@ -2996,7 +2996,7 @@
       </c>
       <c r="F90" t="inlineStr">
         <is>
-          <t>R$ 10.324,00</t>
+          <t>R$ 10.676,00</t>
         </is>
       </c>
     </row>
@@ -3052,7 +3052,7 @@
       </c>
       <c r="F92" t="inlineStr">
         <is>
-          <t>R$ 20.665,00</t>
+          <t>R$ 18.118,00</t>
         </is>
       </c>
     </row>
@@ -4795,7 +4795,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>R$ 6.505,00</t>
+          <t>R$ 18.298,00</t>
         </is>
       </c>
     </row>
@@ -4823,7 +4823,7 @@
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>R$ 29.733,00</t>
+          <t>R$ 28.782,00</t>
         </is>
       </c>
     </row>
@@ -4851,7 +4851,7 @@
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>R$ 5.598,00</t>
+          <t>R$ 8.561,00</t>
         </is>
       </c>
     </row>
@@ -4907,7 +4907,7 @@
       </c>
       <c r="F159" t="inlineStr">
         <is>
-          <t>R$ 13.867,00</t>
+          <t>R$ 31.709,00</t>
         </is>
       </c>
     </row>
@@ -4935,7 +4935,7 @@
       </c>
       <c r="F160" t="inlineStr">
         <is>
-          <t>R$ 7.856,00</t>
+          <t>R$ 8.824,00</t>
         </is>
       </c>
     </row>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="F161" t="inlineStr">
         <is>
-          <t>R$ 33.695,00</t>
+          <t>R$ 17.541,00</t>
         </is>
       </c>
     </row>
@@ -5019,7 +5019,7 @@
       </c>
       <c r="F163" t="inlineStr">
         <is>
-          <t>R$ 32.157,00</t>
+          <t>R$ 18.482,00</t>
         </is>
       </c>
     </row>
@@ -5131,7 +5131,7 @@
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>R$ 6.505,00</t>
+          <t>R$ 28.188,00</t>
         </is>
       </c>
     </row>
@@ -5159,7 +5159,7 @@
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>R$ 14.836,00</t>
+          <t>R$ 41.676,00</t>
         </is>
       </c>
     </row>
@@ -5187,7 +5187,7 @@
       </c>
       <c r="F169" t="inlineStr">
         <is>
-          <t>R$ 14.825,00</t>
+          <t>R$ 14.242,00</t>
         </is>
       </c>
     </row>
@@ -5271,7 +5271,7 @@
       </c>
       <c r="F172" t="inlineStr">
         <is>
-          <t>R$ 30.004,00</t>
+          <t>R$ 30.953,00</t>
         </is>
       </c>
     </row>
@@ -5383,7 +5383,7 @@
       </c>
       <c r="F176" t="inlineStr">
         <is>
-          <t>R$ 9.699,00</t>
+          <t>R$ 7.684,00</t>
         </is>
       </c>
     </row>
@@ -5411,7 +5411,7 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>R$ 6.505,00</t>
+          <t>R$ 13.538,00</t>
         </is>
       </c>
     </row>
@@ -5467,7 +5467,7 @@
       </c>
       <c r="F179" t="inlineStr">
         <is>
-          <t>R$ 5.598,00</t>
+          <t>R$ 8.561,00</t>
         </is>
       </c>
     </row>
@@ -5551,7 +5551,7 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>R$ 12.982,00</t>
+          <t>R$ 36.186,00</t>
         </is>
       </c>
     </row>
@@ -5579,7 +5579,7 @@
       </c>
       <c r="F183" t="inlineStr">
         <is>
-          <t>R$ 11.196,00</t>
+          <t>R$ 9.632,00</t>
         </is>
       </c>
     </row>
@@ -5607,7 +5607,7 @@
       </c>
       <c r="F184" t="inlineStr">
         <is>
-          <t>R$ 9.699,00</t>
+          <t>R$ 7.684,00</t>
         </is>
       </c>
     </row>
@@ -5663,7 +5663,7 @@
       </c>
       <c r="F186" t="inlineStr">
         <is>
-          <t>R$ 9.409,00</t>
+          <t>R$ 11.289,00</t>
         </is>
       </c>
     </row>
@@ -5719,7 +5719,7 @@
       </c>
       <c r="F188" t="inlineStr">
         <is>
-          <t>R$ 13.996,00</t>
+          <t>R$ 10.680,00</t>
         </is>
       </c>
     </row>
@@ -5775,7 +5775,7 @@
       </c>
       <c r="F190" t="inlineStr">
         <is>
-          <t>R$ 7.962,00</t>
+          <t>R$ 15.161,00</t>
         </is>
       </c>
     </row>
@@ -5803,7 +5803,7 @@
       </c>
       <c r="F191" t="inlineStr">
         <is>
-          <t>R$ 10.662,00</t>
+          <t>R$ 21.397,00</t>
         </is>
       </c>
     </row>
@@ -5831,7 +5831,7 @@
       </c>
       <c r="F192" t="inlineStr">
         <is>
-          <t>R$ 17.054,00</t>
+          <t>R$ 20.683,00</t>
         </is>
       </c>
     </row>
@@ -5887,7 +5887,7 @@
       </c>
       <c r="F194" t="inlineStr">
         <is>
-          <t>R$ 10.880,00</t>
+          <t>R$ 20.217,00</t>
         </is>
       </c>
     </row>
@@ -5915,7 +5915,7 @@
       </c>
       <c r="F195" t="inlineStr">
         <is>
-          <t>R$ 38.334,00</t>
+          <t>R$ 71.991,00</t>
         </is>
       </c>
     </row>
@@ -5943,7 +5943,7 @@
       </c>
       <c r="F196" t="inlineStr">
         <is>
-          <t>R$ 19.155,00</t>
+          <t>R$ 9.353,00</t>
         </is>
       </c>
     </row>
@@ -5971,7 +5971,7 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>R$ 12.982,00</t>
+          <t>R$ 36.186,00</t>
         </is>
       </c>
     </row>
@@ -5999,7 +5999,7 @@
       </c>
       <c r="F198" t="inlineStr">
         <is>
-          <t>R$ 16.615,00</t>
+          <t>R$ 14.437,00</t>
         </is>
       </c>
     </row>
@@ -6083,7 +6083,7 @@
       </c>
       <c r="F201" t="inlineStr">
         <is>
-          <t>R$ 34.123,00</t>
+          <t>R$ 26.597,00</t>
         </is>
       </c>
     </row>
@@ -6139,7 +6139,7 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>R$ 19.155,00</t>
+          <t>R$ 10.774,00</t>
         </is>
       </c>
     </row>
@@ -6167,7 +6167,7 @@
       </c>
       <c r="F204" t="inlineStr">
         <is>
-          <t>R$ 11.793,00</t>
+          <t>R$ 12.445,00</t>
         </is>
       </c>
     </row>
@@ -6195,7 +6195,7 @@
       </c>
       <c r="F205" t="inlineStr">
         <is>
-          <t>R$ 13.864,00</t>
+          <t>R$ 16.297,00</t>
         </is>
       </c>
     </row>
@@ -6251,7 +6251,7 @@
       </c>
       <c r="F207" t="inlineStr">
         <is>
-          <t>R$ 9.409,00</t>
+          <t>R$ 8.553,00</t>
         </is>
       </c>
     </row>
@@ -6279,7 +6279,7 @@
       </c>
       <c r="F208" t="inlineStr">
         <is>
-          <t>R$ 6.982,00</t>
+          <t>R$ 10.176,00</t>
         </is>
       </c>
     </row>
@@ -6307,7 +6307,7 @@
       </c>
       <c r="F209" t="inlineStr">
         <is>
-          <t>R$ 56.161,00</t>
+          <t>R$ 17.766,00</t>
         </is>
       </c>
     </row>
@@ -6335,7 +6335,7 @@
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>R$ 12.982,00</t>
+          <t>R$ 36.186,00</t>
         </is>
       </c>
     </row>
@@ -6363,7 +6363,7 @@
       </c>
       <c r="F211" t="inlineStr">
         <is>
-          <t>R$ 17.829,00</t>
+          <t>R$ 19.582,00</t>
         </is>
       </c>
     </row>
@@ -6531,7 +6531,7 @@
       </c>
       <c r="F217" t="inlineStr">
         <is>
-          <t>R$ 9.409,00</t>
+          <t>R$ 11.289,00</t>
         </is>
       </c>
     </row>
@@ -6587,7 +6587,7 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>R$ 13.305,00</t>
+          <t>R$ 28.931,00</t>
         </is>
       </c>
     </row>
@@ -6671,7 +6671,7 @@
       </c>
       <c r="F222" t="inlineStr">
         <is>
-          <t>R$ 23.663,00</t>
+          <t>R$ 22.924,00</t>
         </is>
       </c>
     </row>
@@ -6699,7 +6699,7 @@
       </c>
       <c r="F223" t="inlineStr">
         <is>
-          <t>R$ 9.544,00</t>
+          <t>R$ 19.944,00</t>
         </is>
       </c>
     </row>
@@ -6755,7 +6755,7 @@
       </c>
       <c r="F225" t="inlineStr">
         <is>
-          <t>R$ 5.598,00</t>
+          <t>R$ 6.266,00</t>
         </is>
       </c>
     </row>
@@ -6783,7 +6783,7 @@
       </c>
       <c r="F226" t="inlineStr">
         <is>
-          <t>R$ 14.608,00</t>
+          <t>R$ 12.503,00</t>
         </is>
       </c>
     </row>
@@ -6811,7 +6811,7 @@
       </c>
       <c r="F227" t="inlineStr">
         <is>
-          <t>R$ 35.147,00</t>
+          <t>R$ 39.399,00</t>
         </is>
       </c>
     </row>
@@ -6839,7 +6839,7 @@
       </c>
       <c r="F228" t="inlineStr">
         <is>
-          <t>R$ 10.324,00</t>
+          <t>R$ 22.458,00</t>
         </is>
       </c>
     </row>
@@ -7007,7 +7007,7 @@
       </c>
       <c r="F234" t="inlineStr">
         <is>
-          <t>R$ 27.406,00</t>
+          <t>R$ 10.956,00</t>
         </is>
       </c>
     </row>
@@ -7035,7 +7035,7 @@
       </c>
       <c r="F235" t="inlineStr">
         <is>
-          <t>R$ 34.123,00</t>
+          <t>R$ 21.648,00</t>
         </is>
       </c>
     </row>
@@ -7063,7 +7063,7 @@
       </c>
       <c r="F236" t="inlineStr">
         <is>
-          <t>R$ 52.240,00</t>
+          <t>R$ 26.471,00</t>
         </is>
       </c>
     </row>
@@ -7119,7 +7119,7 @@
       </c>
       <c r="F238" t="inlineStr">
         <is>
-          <t>R$ 10.819,00</t>
+          <t>R$ 9.727,00</t>
         </is>
       </c>
     </row>
@@ -7147,7 +7147,7 @@
       </c>
       <c r="F239" t="inlineStr">
         <is>
-          <t>R$ 21.195,00</t>
+          <t>R$ 37.124,00</t>
         </is>
       </c>
     </row>
@@ -7175,7 +7175,7 @@
       </c>
       <c r="F240" t="inlineStr">
         <is>
-          <t>R$ 11.196,00</t>
+          <t>R$ 9.679,00</t>
         </is>
       </c>
     </row>
@@ -7231,7 +7231,7 @@
       </c>
       <c r="F242" t="inlineStr">
         <is>
-          <t>R$ 10.019,00</t>
+          <t>R$ 9.333,00</t>
         </is>
       </c>
     </row>
@@ -7259,7 +7259,7 @@
       </c>
       <c r="F243" t="inlineStr">
         <is>
-          <t>R$ 15.094,00</t>
+          <t>R$ 9.808,00</t>
         </is>
       </c>
     </row>
@@ -7287,7 +7287,7 @@
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>R$ 6.505,00</t>
+          <t>R$ 13.538,00</t>
         </is>
       </c>
     </row>
@@ -7343,7 +7343,7 @@
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>R$ 42.228,00</t>
+          <t>R$ 27.528,00</t>
         </is>
       </c>
     </row>
@@ -7371,7 +7371,7 @@
       </c>
       <c r="F247" t="inlineStr">
         <is>
-          <t>R$ 12.568,00</t>
+          <t>R$ 5.202,00</t>
         </is>
       </c>
     </row>
@@ -7399,7 +7399,7 @@
       </c>
       <c r="F248" t="inlineStr">
         <is>
-          <t>R$ 30.538,00</t>
+          <t>R$ 19.392,00</t>
         </is>
       </c>
     </row>
@@ -9058,7 +9058,7 @@
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>R$ 12.982,00</t>
+          <t>R$ 32.854,00</t>
         </is>
       </c>
     </row>
@@ -9114,7 +9114,7 @@
       </c>
       <c r="F310" t="inlineStr">
         <is>
-          <t>R$ 9.656,00</t>
+          <t>R$ 13.270,00</t>
         </is>
       </c>
     </row>
@@ -9142,7 +9142,7 @@
       </c>
       <c r="F311" t="inlineStr">
         <is>
-          <t>R$ 6.505,00</t>
+          <t>R$ 11.289,00</t>
         </is>
       </c>
     </row>
@@ -9170,7 +9170,7 @@
       </c>
       <c r="F312" t="inlineStr">
         <is>
-          <t>R$ 30.537,00</t>
+          <t>R$ 23.319,00</t>
         </is>
       </c>
     </row>
@@ -9226,7 +9226,7 @@
       </c>
       <c r="F314" t="inlineStr">
         <is>
-          <t>R$ 7.678,00</t>
+          <t>R$ 8.910,00</t>
         </is>
       </c>
     </row>
@@ -9282,7 +9282,7 @@
       </c>
       <c r="F316" t="inlineStr">
         <is>
-          <t>R$ 13.864,00</t>
+          <t>R$ 15.899,00</t>
         </is>
       </c>
     </row>
@@ -9366,7 +9366,7 @@
       </c>
       <c r="F319" t="inlineStr">
         <is>
-          <t>R$ 20.522,00</t>
+          <t>R$ 9.693,00</t>
         </is>
       </c>
     </row>
@@ -9394,7 +9394,7 @@
       </c>
       <c r="F320" t="inlineStr">
         <is>
-          <t>R$ 6.505,00</t>
+          <t>R$ 27.806,00</t>
         </is>
       </c>
     </row>
@@ -9450,7 +9450,7 @@
       </c>
       <c r="F322" t="inlineStr">
         <is>
-          <t>R$ 7.752,00</t>
+          <t>R$ 8.016,00</t>
         </is>
       </c>
     </row>
@@ -9478,7 +9478,7 @@
       </c>
       <c r="F323" t="inlineStr">
         <is>
-          <t>R$ 9.544,00</t>
+          <t>R$ 26.156,00</t>
         </is>
       </c>
     </row>
@@ -9534,7 +9534,7 @@
       </c>
       <c r="F325" t="inlineStr">
         <is>
-          <t>R$ 10.270,00</t>
+          <t>R$ 14.173,00</t>
         </is>
       </c>
     </row>
@@ -9562,7 +9562,7 @@
       </c>
       <c r="F326" t="inlineStr">
         <is>
-          <t>R$ 7.678,00</t>
+          <t>R$ 8.283,00</t>
         </is>
       </c>
     </row>
@@ -9618,7 +9618,7 @@
       </c>
       <c r="F328" t="inlineStr">
         <is>
-          <t>R$ 6.505,00</t>
+          <t>R$ 25.616,00</t>
         </is>
       </c>
     </row>
@@ -9674,7 +9674,7 @@
       </c>
       <c r="F330" t="inlineStr">
         <is>
-          <t>R$ 10.967,00</t>
+          <t>R$ 32.501,00</t>
         </is>
       </c>
     </row>
@@ -9730,7 +9730,7 @@
       </c>
       <c r="F332" t="inlineStr">
         <is>
-          <t>R$ 24.182,00</t>
+          <t>R$ 11.194,00</t>
         </is>
       </c>
     </row>
@@ -9758,7 +9758,7 @@
       </c>
       <c r="F333" t="inlineStr">
         <is>
-          <t>R$ 14.495,00</t>
+          <t>R$ 24.772,00</t>
         </is>
       </c>
     </row>
@@ -9786,7 +9786,7 @@
       </c>
       <c r="F334" t="inlineStr">
         <is>
-          <t>R$ 8.865,00</t>
+          <t>R$ 4.727,00</t>
         </is>
       </c>
     </row>
@@ -9814,7 +9814,7 @@
       </c>
       <c r="F335" t="inlineStr">
         <is>
-          <t>R$ 37.363,00</t>
+          <t>R$ 15.950,00</t>
         </is>
       </c>
     </row>
@@ -9954,7 +9954,7 @@
       </c>
       <c r="F340" t="inlineStr">
         <is>
-          <t>R$ 6.505,00</t>
+          <t>R$ 24.466,00</t>
         </is>
       </c>
     </row>
@@ -9982,7 +9982,7 @@
       </c>
       <c r="F341" t="inlineStr">
         <is>
-          <t>R$ 14.608,00</t>
+          <t>R$ 21.779,00</t>
         </is>
       </c>
     </row>
@@ -10010,7 +10010,7 @@
       </c>
       <c r="F342" t="inlineStr">
         <is>
-          <t>R$ 10.967,00</t>
+          <t>R$ 15.020,00</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix premium variant mismatches: penalize GTi/GTS/Turbo when not in input, handle 1000cc=1.0L displacement equivalence
GOL 16V no longer matches GTi 2000 16V (R$36K->R$13K), GOL 1000 no longer matches GTi 2.0 (R$28K->R$8K)
</commit_message>
<xml_diff>
--- a/lotes_leilao_com_fipe.xlsx
+++ b/lotes_leilao_com_fipe.xlsx
@@ -1960,7 +1960,7 @@
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>R$ 8.553,00</t>
+          <t>R$ 12.430,00</t>
         </is>
       </c>
     </row>
@@ -1988,7 +1988,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>R$ 18.298,00</t>
+          <t>R$ 13.305,00</t>
         </is>
       </c>
     </row>
@@ -2072,7 +2072,7 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>R$ 8.553,00</t>
+          <t>R$ 12.430,00</t>
         </is>
       </c>
     </row>
@@ -2268,7 +2268,7 @@
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>R$ 8.588,00</t>
+          <t>R$ 8.780,00</t>
         </is>
       </c>
     </row>
@@ -4795,7 +4795,7 @@
       </c>
       <c r="F155" t="inlineStr">
         <is>
-          <t>R$ 18.298,00</t>
+          <t>R$ 13.305,00</t>
         </is>
       </c>
     </row>
@@ -5411,7 +5411,7 @@
       </c>
       <c r="F177" t="inlineStr">
         <is>
-          <t>R$ 13.538,00</t>
+          <t>R$ 13.305,00</t>
         </is>
       </c>
     </row>
@@ -5551,7 +5551,7 @@
       </c>
       <c r="F182" t="inlineStr">
         <is>
-          <t>R$ 36.186,00</t>
+          <t>R$ 12.982,00</t>
         </is>
       </c>
     </row>
@@ -5971,7 +5971,7 @@
       </c>
       <c r="F197" t="inlineStr">
         <is>
-          <t>R$ 36.186,00</t>
+          <t>R$ 12.982,00</t>
         </is>
       </c>
     </row>
@@ -6139,7 +6139,7 @@
       </c>
       <c r="F203" t="inlineStr">
         <is>
-          <t>R$ 10.774,00</t>
+          <t>R$ 11.942,00</t>
         </is>
       </c>
     </row>
@@ -6335,7 +6335,7 @@
       </c>
       <c r="F210" t="inlineStr">
         <is>
-          <t>R$ 36.186,00</t>
+          <t>R$ 12.982,00</t>
         </is>
       </c>
     </row>
@@ -6587,7 +6587,7 @@
       </c>
       <c r="F219" t="inlineStr">
         <is>
-          <t>R$ 28.931,00</t>
+          <t>R$ 8.488,00</t>
         </is>
       </c>
     </row>
@@ -7091,7 +7091,7 @@
       </c>
       <c r="F237" t="inlineStr">
         <is>
-          <t>R$ 35.871,00</t>
+          <t>R$ 33.790,00</t>
         </is>
       </c>
     </row>
@@ -7287,7 +7287,7 @@
       </c>
       <c r="F244" t="inlineStr">
         <is>
-          <t>R$ 13.538,00</t>
+          <t>R$ 13.305,00</t>
         </is>
       </c>
     </row>
@@ -7343,7 +7343,7 @@
       </c>
       <c r="F246" t="inlineStr">
         <is>
-          <t>R$ 27.528,00</t>
+          <t>R$ 30.799,00</t>
         </is>
       </c>
     </row>
@@ -9002,7 +9002,7 @@
       </c>
       <c r="F306" t="inlineStr">
         <is>
-          <t>R$ 7.899,00</t>
+          <t>R$ 5.293,00</t>
         </is>
       </c>
     </row>
@@ -9058,7 +9058,7 @@
       </c>
       <c r="F308" t="inlineStr">
         <is>
-          <t>R$ 32.854,00</t>
+          <t>R$ 12.982,00</t>
         </is>
       </c>
     </row>

</xml_diff>